<commit_message>
Actualización automática de catálogo y fotos
</commit_message>
<xml_diff>
--- a/catalogo.xlsx
+++ b/catalogo.xlsx
@@ -13,14 +13,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="1yG/eLgU41PGmotHI2ElPk+sJpWFlJirXKy51IoTgJA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="qG4wC4nVVHGvzzWMC3Ah1xFPXdV+uqPdFbqYEsVd6+8="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="206">
   <si>
     <t>nombre</t>
   </si>
@@ -115,6 +115,9 @@
     <t>chicago dorado meta.jpg</t>
   </si>
   <si>
+    <t>chicago dorado meta 2.jpg</t>
+  </si>
+  <si>
     <t>Chicago Crochet Blanco Perla</t>
   </si>
   <si>
@@ -172,12 +175,12 @@
     <t>Kioto Negro</t>
   </si>
   <si>
+    <t>kioto negro puesto 1.jpg</t>
+  </si>
+  <si>
     <t>kioto negro fb.jpg</t>
   </si>
   <si>
-    <t>kioto negro puesto 1.jpg</t>
-  </si>
-  <si>
     <t>Kioto Morado</t>
   </si>
   <si>
@@ -226,12 +229,12 @@
     <t>San Francisco Cotton Camel</t>
   </si>
   <si>
+    <t>sf camel 2.jpg</t>
+  </si>
+  <si>
     <t>sf cotton camel.jpg</t>
   </si>
   <si>
-    <t>sf camel 2.jpg</t>
-  </si>
-  <si>
     <t>San Francisco Cotton Vainilla</t>
   </si>
   <si>
@@ -313,15 +316,15 @@
     <t>Mini Madrid Cotton Verde</t>
   </si>
   <si>
+    <t>mini madrid verde 3.jpg</t>
+  </si>
+  <si>
+    <t>mini madrid verde.jpg</t>
+  </si>
+  <si>
     <t>mini madrid verde fb.jpg</t>
   </si>
   <si>
-    <t>mini madrid verde.jpg</t>
-  </si>
-  <si>
-    <t>mini madrid verde 3.jpg</t>
-  </si>
-  <si>
     <t>Mini Madrid Cotton Fucsia</t>
   </si>
   <si>
@@ -349,12 +352,12 @@
     <t>Madrid Cotton Chocolate</t>
   </si>
   <si>
+    <t>madrid chocolate 2.jpg</t>
+  </si>
+  <si>
     <t>madrid chocolate fb.jpg</t>
   </si>
   <si>
-    <t>madrid chocolate 2.jpg</t>
-  </si>
-  <si>
     <t>Huesca Cotton Chocolate</t>
   </si>
   <si>
@@ -602,6 +605,21 @@
   </si>
   <si>
     <t>Choker beige.jpg</t>
+  </si>
+  <si>
+    <t>Choker Flor</t>
+  </si>
+  <si>
+    <t>Flor</t>
+  </si>
+  <si>
+    <t>choker flor.jpg</t>
+  </si>
+  <si>
+    <t>choker flor 2.jpg</t>
+  </si>
+  <si>
+    <t>choker flor 3.jpg</t>
   </si>
   <si>
     <t>Conjunto Paris y Milan</t>
@@ -661,7 +679,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -670,6 +688,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -783,7 +804,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I47" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I48" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="9">
     <tableColumn name="nombre" id="1"/>
     <tableColumn name="tipo" id="2"/>
@@ -800,7 +821,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A70:I73" displayName="Table_10" name="Table_10" id="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A71:I75" displayName="Table_10" name="Table_10" id="10">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -826,7 +847,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="C1:C18" displayName="Table_12" name="Table_12" id="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="C1:C19" displayName="Table_12" name="Table_12" id="12">
   <tableColumns count="1">
     <tableColumn name="categoría" id="1"/>
   </tableColumns>
@@ -835,7 +856,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A48:I48" displayName="Table_2" name="Table_2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A49:I49" displayName="Table_2" name="Table_2" id="2">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -852,7 +873,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A49:I49" displayName="Table_3" name="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A50:I50" displayName="Table_3" name="Table_3" id="3">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -869,7 +890,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A50:I50" displayName="Table_4" name="Table_4" id="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A51:I51" displayName="Table_4" name="Table_4" id="4">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -886,7 +907,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A51:I59" displayName="Table_5" name="Table_5" id="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A52:I60" displayName="Table_5" name="Table_5" id="5">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -903,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A60:I60" displayName="Table_6" name="Table_6" id="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A61:I61" displayName="Table_6" name="Table_6" id="6">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -920,7 +941,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A61:I61" displayName="Table_7" name="Table_7" id="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A62:I62" displayName="Table_7" name="Table_7" id="7">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -937,7 +958,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A62:I68" displayName="Table_8" name="Table_8" id="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A63:I69" displayName="Table_8" name="Table_8" id="8">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -954,7 +975,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A69:I69" displayName="Table_9" name="Table_9" id="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A70:I70" displayName="Table_9" name="Table_9" id="9">
   <tableColumns count="9">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -1369,7 +1390,7 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>10</v>
@@ -1378,10 +1399,10 @@
         <v>11</v>
       </c>
       <c r="D9" s="3">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1389,360 +1410,359 @@
       <c r="I9" s="1"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" ht="14.25" customHeight="1">
+      <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="B11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="D11" s="3">
         <v>30.0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H11" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>34</v>
+      <c r="C12" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="D12" s="3">
         <v>30.0</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>34</v>
+      <c r="C13" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="D13" s="3">
         <v>30.0</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>46</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>34</v>
+      <c r="C14" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="D14" s="3">
         <v>30.0</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G14" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3">
         <v>30.0</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" ht="15.0" customHeight="1">
+    <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D16" s="3">
         <v>30.0</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
     <row r="17" ht="15.0" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" s="3">
         <v>30.0</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F17" s="2"/>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" ht="14.25" customHeight="1">
+    <row r="18" ht="15.0" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="3">
-        <v>25.0</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="F18" s="2"/>
       <c r="I18" s="1"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D19" s="3">
         <v>25.0</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F19" s="2"/>
       <c r="I19" s="1"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="F20" s="2"/>
       <c r="I20" s="1"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="3">
-        <v>25.0</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="F21" s="2"/>
       <c r="I21" s="1"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" s="3">
         <v>25.0</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="F22" s="2"/>
       <c r="I22" s="1"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D23" s="3">
         <v>25.0</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="1"/>
+        <v>66</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="I23" s="1"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D24" s="3">
         <v>25.0</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D25" s="3">
         <v>25.0</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="E25" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D26" s="3">
         <v>25.0</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="1"/>
@@ -1750,40 +1770,39 @@
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D27" s="3">
         <v>25.0</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F27" s="2"/>
+        <v>76</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1792,19 +1811,19 @@
     </row>
     <row r="29" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D29" s="3">
-        <v>40.0</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -1813,107 +1832,107 @@
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D30" s="3">
         <v>40.0</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>86</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" s="3">
+        <v>40.0</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D31" s="3">
-        <v>25.0</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F31" s="2"/>
-      <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
     </row>
     <row r="32" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D32" s="3">
         <v>25.0</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
+      <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D33" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D34" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -1922,65 +1941,64 @@
     </row>
     <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D35" s="3">
         <v>20.0</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>99</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D36" s="3">
         <v>20.0</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+        <v>98</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>100</v>
+      </c>
       <c r="I36" s="1"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D37" s="3">
         <v>20.0</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
@@ -1989,45 +2007,43 @@
     </row>
     <row r="38" ht="14.25" customHeight="1">
       <c r="A38" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D38" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D38" s="3">
-        <v>25.0</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>107</v>
-      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D39" s="3">
         <v>25.0</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
@@ -2035,40 +2051,41 @@
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D40" s="3">
         <v>25.0</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
+        <v>110</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>111</v>
+      </c>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
     </row>
     <row r="41" ht="14.25" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D41" s="3">
         <v>25.0</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
@@ -2077,19 +2094,19 @@
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D42" s="3">
         <v>25.0</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
@@ -2098,19 +2115,19 @@
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D43" s="3">
         <v>25.0</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
@@ -2119,19 +2136,19 @@
     </row>
     <row r="44" ht="14.25" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D44" s="3">
         <v>25.0</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
@@ -2140,84 +2157,84 @@
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D45" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D45" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>125</v>
-      </c>
+      <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D46" s="3">
         <v>30.0</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="F46" s="2"/>
+        <v>125</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
     </row>
     <row r="47" ht="14.25" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D47" s="3">
         <v>30.0</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="F47" s="1"/>
+        <v>129</v>
+      </c>
+      <c r="F47" s="2"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D48" s="3">
         <v>30.0</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
@@ -2226,19 +2243,19 @@
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D49" s="3">
         <v>30.0</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
@@ -2247,106 +2264,106 @@
     </row>
     <row r="50" ht="14.25" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D50" s="3">
         <v>30.0</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="F50" s="2"/>
+        <v>135</v>
+      </c>
+      <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D51" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="E51" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D51" s="3">
-        <v>13.0</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="F51" s="1"/>
+      <c r="F51" s="2"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D52" s="3">
         <v>13.0</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
       <c r="I52" s="1"/>
     </row>
     <row r="53" ht="14.25" customHeight="1">
       <c r="A53" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D53" s="3">
         <v>13.0</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F53" s="1"/>
-      <c r="G53" s="1"/>
-      <c r="H53" s="1"/>
+        <v>143</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>145</v>
+      </c>
       <c r="I53" s="1"/>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D54" s="3">
         <v>13.0</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
@@ -2355,40 +2372,40 @@
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D55" s="3">
         <v>13.0</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F55" s="2"/>
+        <v>149</v>
+      </c>
+      <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
     </row>
     <row r="56" ht="14.25" customHeight="1">
       <c r="A56" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D56" s="3">
         <v>13.0</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="1"/>
@@ -2397,32 +2414,34 @@
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D57" s="3">
         <v>13.0</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F57" s="2"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
       <c r="I57" s="1"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="C58" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D58" s="3">
         <v>13.0</v>
@@ -2435,32 +2454,32 @@
     </row>
     <row r="59" ht="14.25" customHeight="1">
       <c r="A59" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D59" s="3">
+        <v>13.0</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="D59" s="3">
-        <v>15.0</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="F59" s="2"/>
       <c r="I59" s="1"/>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D60" s="3">
         <v>15.0</v>
@@ -2468,39 +2487,39 @@
       <c r="E60" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="F60" s="2" t="s">
-        <v>161</v>
-      </c>
+      <c r="F60" s="2"/>
       <c r="I60" s="1"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D61" s="3">
         <v>15.0</v>
       </c>
       <c r="E61" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F61" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F61" s="2"/>
       <c r="I61" s="1"/>
     </row>
     <row r="62" ht="14.25" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D62" s="3">
         <v>15.0</v>
@@ -2513,13 +2532,13 @@
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D63" s="3">
         <v>15.0</v>
@@ -2528,25 +2547,23 @@
         <v>164</v>
       </c>
       <c r="F63" s="2"/>
-      <c r="G63" s="1"/>
-      <c r="H63" s="1"/>
       <c r="I63" s="1"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D64" s="3">
         <v>15.0</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F64" s="2"/>
       <c r="G64" s="1"/>
@@ -2555,88 +2572,88 @@
     </row>
     <row r="65" ht="14.25" customHeight="1">
       <c r="A65" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D65" s="3">
         <v>15.0</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>171</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="F65" s="2"/>
+      <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D66" s="3">
         <v>15.0</v>
       </c>
       <c r="E66" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G66" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D67" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F67" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D67" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F67" s="2"/>
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
     </row>
     <row r="68" ht="14.25" customHeight="1">
       <c r="A68" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D68" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="E68" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D68" s="3">
-        <v>10.0</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="F68" s="2"/>
       <c r="G68" s="1"/>
@@ -2645,32 +2662,34 @@
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D69" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D69" s="3">
-        <v>12.0</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>181</v>
-      </c>
       <c r="F69" s="2"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
       <c r="I69" s="1"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D70" s="3">
         <v>12.0</v>
@@ -2683,40 +2702,38 @@
     </row>
     <row r="71" ht="14.25" customHeight="1">
       <c r="A71" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D71" s="3">
         <v>12.0</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F71" s="2"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
       <c r="I71" s="1"/>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D72" s="3">
         <v>12.0</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F72" s="2"/>
       <c r="G72" s="4"/>
@@ -2725,55 +2742,99 @@
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D73" s="3">
+        <v>12.0</v>
+      </c>
+      <c r="E73" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C73" s="2" t="s">
+      <c r="F73" s="2"/>
+      <c r="G73" s="4"/>
+      <c r="H73" s="4"/>
+      <c r="I73" s="1"/>
+    </row>
+    <row r="74" ht="14.25" customHeight="1">
+      <c r="A74" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="D73" s="3">
+      <c r="B74" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D74" s="3">
         <v>13.0</v>
       </c>
-      <c r="E73" s="2" t="s">
+      <c r="E74" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G74" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="H74" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="I74" s="1"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D75" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H75" s="5"/>
+      <c r="I75" s="1"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="F73" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G73" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="H73" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="I73" s="1"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="D74" s="3">
+      <c r="D76" s="3">
         <v>18.0</v>
       </c>
-      <c r="E74" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="3"/>
-    </row>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
+      <c r="E76" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="3"/>
+    </row>
     <row r="82" ht="14.25" customHeight="1"/>
     <row r="83" ht="14.25" customHeight="1"/>
     <row r="84" ht="14.25" customHeight="1"/>
@@ -3698,12 +3759,14 @@
     <row r="1003" ht="14.25" customHeight="1"/>
     <row r="1004" ht="14.25" customHeight="1"/>
     <row r="1005" ht="14.25" customHeight="1"/>
+    <row r="1006" ht="14.25" customHeight="1"/>
+    <row r="1007" ht="14.25" customHeight="1"/>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C75">
-      <formula1>datos!$C$2:$C$18</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C77">
+      <formula1>datos!$C$2:$C$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B75">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B77">
       <formula1>datos!$A$2:$A$6</formula1>
     </dataValidation>
   </dataValidations>
@@ -3740,7 +3803,7 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3756,97 +3819,101 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="C7" s="2" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="C8" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="C9" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="C10" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="C11" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="C12" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="C13" s="2" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="C14" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="C15" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="C16" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="C17" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="C18" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="19" ht="14.25" customHeight="1"/>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25" customHeight="1">
+      <c r="C19" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
     <row r="20" ht="14.25" customHeight="1"/>
     <row r="21" ht="14.25" customHeight="1"/>
     <row r="22" ht="14.25" customHeight="1"/>

</xml_diff>